<commit_message>
chore: atualizacao SICARD 2026-10-22 13:08
</commit_message>
<xml_diff>
--- a/documentacao/matrizes/Modelo_Matriz_Criterios_Premissas_SLT.xlsx
+++ b/documentacao/matrizes/Modelo_Matriz_Criterios_Premissas_SLT.xlsx
@@ -458,6 +458,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -521,7 +522,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Coluna 'Etapa': use apenas um dos valores da lista — Elegibilidade territorial, Favorabilidade territorial em grade e da rede, Ajuste por atributos do objeto de demanda.</t>
+          <t>Coluna 'Etapa': use apenas um dos valores da lista — Elegibilidade territorial, Favorabilidade territorial — município e rede rodoviária, Priorização de demandas por atributos.</t>
         </is>
       </c>
     </row>
@@ -609,6 +610,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
@@ -715,7 +717,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Favorabilidade territorial em grade e da rede</t>
+          <t>Favorabilidade territorial — município e rede rodoviária</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -747,7 +749,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ajuste por atributos do objeto de demanda</t>
+          <t>Priorização de demandas por atributos</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">

</xml_diff>